<commit_message>
MUDANÇA SIMPLES PARA AJUSTE CUSTO P/ CABECA POR FAZENDA
</commit_message>
<xml_diff>
--- a/Diarias/CustoPcabeça.xlsx
+++ b/Diarias/CustoPcabeça.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henrique.santos\orcamento2027\budgetflow-insights\Diarias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64591AA1-8925-453A-80EE-6428B95C5EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6082FC5D-A4D7-40BA-886A-4020C069598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5B15AADF-5E25-4D61-AF8C-F30613BBBE1E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5B15AADF-5E25-4D61-AF8C-F30613BBBE1E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="GERAL" sheetId="1" r:id="rId1"/>
+    <sheet name="FAZENDAS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,12 +40,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
   <si>
     <t>Orçado</t>
   </si>
   <si>
     <t>Realizado</t>
+  </si>
+  <si>
+    <t>BANDEIRANTES - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>PORTEIRAS - PECUÁRIA</t>
   </si>
 </sst>
 </file>
@@ -635,4 +642,234 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C491CF5F-31A9-4DE6-8F5D-68C91161E64E}">
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D1" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E1" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>132.31644803131445</v>
+      </c>
+      <c r="D2">
+        <v>159.43677698882601</v>
+      </c>
+      <c r="E2">
+        <v>194.38455111090798</v>
+      </c>
+      <c r="F2">
+        <v>153.9176320360703</v>
+      </c>
+      <c r="G2">
+        <v>155.69229896499075</v>
+      </c>
+      <c r="H2">
+        <v>123.71875153285998</v>
+      </c>
+      <c r="I2">
+        <v>124.0568670599384</v>
+      </c>
+      <c r="J2">
+        <v>124.1358648427837</v>
+      </c>
+      <c r="K2">
+        <v>128.51127179466201</v>
+      </c>
+      <c r="L2">
+        <v>105.01595263790503</v>
+      </c>
+      <c r="M2">
+        <v>112.60064933711858</v>
+      </c>
+      <c r="N2">
+        <v>114.71338906302819</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>120</v>
+      </c>
+      <c r="D3">
+        <v>120</v>
+      </c>
+      <c r="E3">
+        <v>120</v>
+      </c>
+      <c r="F3">
+        <v>120</v>
+      </c>
+      <c r="G3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E6" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F6" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G6" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H6" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I6" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L6" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M6" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>120</v>
+      </c>
+      <c r="D7">
+        <v>120</v>
+      </c>
+      <c r="E7">
+        <v>120</v>
+      </c>
+      <c r="F7">
+        <v>120</v>
+      </c>
+      <c r="G7">
+        <v>120</v>
+      </c>
+      <c r="H7">
+        <v>120</v>
+      </c>
+      <c r="I7">
+        <v>120</v>
+      </c>
+      <c r="J7">
+        <v>120</v>
+      </c>
+      <c r="K7">
+        <v>120</v>
+      </c>
+      <c r="L7">
+        <v>120</v>
+      </c>
+      <c r="M7">
+        <v>120</v>
+      </c>
+      <c r="N7">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>120</v>
+      </c>
+      <c r="D8">
+        <v>120</v>
+      </c>
+      <c r="E8">
+        <v>120</v>
+      </c>
+      <c r="F8">
+        <v>120</v>
+      </c>
+      <c r="G8">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
AJUSTE CUSTO P/ CABECA POR FAZENDA
</commit_message>
<xml_diff>
--- a/Diarias/CustoPcabeça.xlsx
+++ b/Diarias/CustoPcabeça.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henrique.santos\orcamento2027\budgetflow-insights\Diarias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6082FC5D-A4D7-40BA-886A-4020C069598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C2F339-8EA5-4E0A-BFB8-5CC38004B89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5B15AADF-5E25-4D61-AF8C-F30613BBBE1E}"/>
+    <workbookView xWindow="-20520" yWindow="1920" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{5B15AADF-5E25-4D61-AF8C-F30613BBBE1E}"/>
   </bookViews>
   <sheets>
     <sheet name="GERAL" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="12">
   <si>
     <t>Orçado</t>
   </si>
@@ -52,6 +52,30 @@
   </si>
   <si>
     <t>PORTEIRAS - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>CODORA</t>
+  </si>
+  <si>
+    <t>JOIA - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>COVOA - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>VERA CRUZ - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>UNIÃO - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>CANADÁ - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>GOTEJO - PECUÁRIA</t>
+  </si>
+  <si>
+    <t>CENTRO COMERCIAL DE TOUROS</t>
   </si>
 </sst>
 </file>
@@ -646,10 +670,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C491CF5F-31A9-4DE6-8F5D-68C91161E64E}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -745,19 +769,19 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>120</v>
+        <v>117.51060320452403</v>
       </c>
       <c r="D3">
-        <v>120</v>
+        <v>96.255322128851546</v>
       </c>
       <c r="E3">
-        <v>120</v>
+        <v>231.90587172538392</v>
       </c>
       <c r="F3">
-        <v>120</v>
+        <v>167.01511476021645</v>
       </c>
       <c r="G3">
-        <v>120</v>
+        <v>128.70144260924107</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -810,40 +834,40 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>120</v>
+        <v>105.33575220637248</v>
       </c>
       <c r="D7">
-        <v>120</v>
+        <v>118.3888169935386</v>
       </c>
       <c r="E7">
-        <v>120</v>
+        <v>121.59377076462754</v>
       </c>
       <c r="F7">
-        <v>120</v>
+        <v>86.597608118432902</v>
       </c>
       <c r="G7">
-        <v>120</v>
+        <v>105.25928706284229</v>
       </c>
       <c r="H7">
-        <v>120</v>
+        <v>124.17992289743626</v>
       </c>
       <c r="I7">
-        <v>120</v>
+        <v>118.63676634453692</v>
       </c>
       <c r="J7">
-        <v>120</v>
+        <v>144.74364604840943</v>
       </c>
       <c r="K7">
-        <v>120</v>
+        <v>82.779156194032666</v>
       </c>
       <c r="L7">
-        <v>120</v>
+        <v>92.541980769723608</v>
       </c>
       <c r="M7">
-        <v>120</v>
+        <v>102.95114051984925</v>
       </c>
       <c r="N7">
-        <v>120</v>
+        <v>119.94995517600671</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -854,19 +878,891 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>120</v>
+        <v>114.65853658536585</v>
       </c>
       <c r="D8">
-        <v>120</v>
+        <v>91.577235772357724</v>
       </c>
       <c r="E8">
-        <v>120</v>
+        <v>247.75</v>
       </c>
       <c r="F8">
-        <v>120</v>
+        <v>136.6</v>
       </c>
       <c r="G8">
-        <v>120</v>
+        <v>218.28205128205127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D11" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E11" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F11" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G11" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H11" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I11" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L11" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M11" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>77.186823246760198</v>
+      </c>
+      <c r="D12">
+        <v>88.99455321398591</v>
+      </c>
+      <c r="E12">
+        <v>114.0496123064291</v>
+      </c>
+      <c r="F12">
+        <v>96.755628027200345</v>
+      </c>
+      <c r="G12">
+        <v>101.91575873302219</v>
+      </c>
+      <c r="H12">
+        <v>89.397971544206214</v>
+      </c>
+      <c r="I12">
+        <v>110.39998201725541</v>
+      </c>
+      <c r="J12">
+        <v>91.299121319171988</v>
+      </c>
+      <c r="K12">
+        <v>77.092983737216599</v>
+      </c>
+      <c r="L12">
+        <v>72.755455818452774</v>
+      </c>
+      <c r="M12">
+        <v>71.677744546284416</v>
+      </c>
+      <c r="N12">
+        <v>52.779785092262998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>101.39901477832512</v>
+      </c>
+      <c r="D13">
+        <v>95.285092491838952</v>
+      </c>
+      <c r="E13">
+        <v>117.36343852013057</v>
+      </c>
+      <c r="F13">
+        <v>219.5174506828528</v>
+      </c>
+      <c r="G13">
+        <v>160.22056384742953</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D16" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E16" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F16" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G16" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H16" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I16" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L16" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M16" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>81.967726047288537</v>
+      </c>
+      <c r="D17">
+        <v>100.86908775486087</v>
+      </c>
+      <c r="E17">
+        <v>104.91563942647878</v>
+      </c>
+      <c r="F17">
+        <v>85.200294330762574</v>
+      </c>
+      <c r="G17">
+        <v>96.362516011629566</v>
+      </c>
+      <c r="H17">
+        <v>96.564014700411548</v>
+      </c>
+      <c r="I17">
+        <v>87.51505753454272</v>
+      </c>
+      <c r="J17">
+        <v>97.836386735167935</v>
+      </c>
+      <c r="K17">
+        <v>109.60720786679171</v>
+      </c>
+      <c r="L17">
+        <v>103.12067850805155</v>
+      </c>
+      <c r="M17">
+        <v>99.290534660840834</v>
+      </c>
+      <c r="N17">
+        <v>79.333669326733656</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>126.68687062434066</v>
+      </c>
+      <c r="D18">
+        <v>131.32635201573254</v>
+      </c>
+      <c r="E18">
+        <v>146.52121951219513</v>
+      </c>
+      <c r="F18">
+        <v>195.64478493112173</v>
+      </c>
+      <c r="G18">
+        <v>206.34827912851279</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D21" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E21" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F21" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G21" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H21" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I21" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L21" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M21" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N21" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>93.271405415499999</v>
+      </c>
+      <c r="D22">
+        <v>274.28656248325001</v>
+      </c>
+      <c r="E22">
+        <v>154.49494654925002</v>
+      </c>
+      <c r="F22">
+        <v>227.50297205487499</v>
+      </c>
+      <c r="G22">
+        <v>231.42855995000002</v>
+      </c>
+      <c r="H22">
+        <v>609.3973827755002</v>
+      </c>
+      <c r="I22">
+        <v>554.50570473850007</v>
+      </c>
+      <c r="J22">
+        <v>91.112461866749996</v>
+      </c>
+      <c r="K22">
+        <v>208.899421563375</v>
+      </c>
+      <c r="L22">
+        <v>661.08860464124996</v>
+      </c>
+      <c r="M22">
+        <v>56.803146016500001</v>
+      </c>
+      <c r="N22">
+        <v>65.216521416749998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1119.6909090909091</v>
+      </c>
+      <c r="D23">
+        <v>485.21794871794873</v>
+      </c>
+      <c r="E23">
+        <v>225.95652173913044</v>
+      </c>
+      <c r="F23">
+        <v>57.243749999999999</v>
+      </c>
+      <c r="G23">
+        <v>6028.25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D26" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E26" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F26" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G26" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H26" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I26" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L26" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M26" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N26" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>78.139715891997056</v>
+      </c>
+      <c r="D27">
+        <v>110.60134377598123</v>
+      </c>
+      <c r="E27">
+        <v>147.2243052912068</v>
+      </c>
+      <c r="F27">
+        <v>100.90286301985546</v>
+      </c>
+      <c r="G27">
+        <v>105.38508561426156</v>
+      </c>
+      <c r="H27">
+        <v>80.087928587268621</v>
+      </c>
+      <c r="I27">
+        <v>96.571062748500552</v>
+      </c>
+      <c r="J27">
+        <v>104.79523607624515</v>
+      </c>
+      <c r="K27">
+        <v>69.302015154978264</v>
+      </c>
+      <c r="L27">
+        <v>54.231221583825324</v>
+      </c>
+      <c r="M27">
+        <v>54.066382542574814</v>
+      </c>
+      <c r="N27">
+        <v>59.471635043658857</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>117.84140127388535</v>
+      </c>
+      <c r="D28">
+        <v>87.329864724245581</v>
+      </c>
+      <c r="E28">
+        <v>69.330741079597445</v>
+      </c>
+      <c r="F28">
+        <v>61.728559176672384</v>
+      </c>
+      <c r="G28">
+        <v>132.17016574585637</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D31" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E31" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F31" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G31" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H31" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I31" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J31" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K31" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L31" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M31" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N31" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>180.35899086267878</v>
+      </c>
+      <c r="D32">
+        <v>159.54143224046533</v>
+      </c>
+      <c r="E32">
+        <v>226.01029887949903</v>
+      </c>
+      <c r="F32">
+        <v>205.56230347997271</v>
+      </c>
+      <c r="G32">
+        <v>207.7711929611757</v>
+      </c>
+      <c r="H32">
+        <v>235.99392527840561</v>
+      </c>
+      <c r="I32">
+        <v>239.991567331753</v>
+      </c>
+      <c r="J32">
+        <v>231.87727266764534</v>
+      </c>
+      <c r="K32">
+        <v>207.8144821153457</v>
+      </c>
+      <c r="L32">
+        <v>125.03592088083691</v>
+      </c>
+      <c r="M32">
+        <v>124.24140352863459</v>
+      </c>
+      <c r="N32">
+        <v>127.24990152618362</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>185.21895861148198</v>
+      </c>
+      <c r="D33">
+        <v>160.63023679417122</v>
+      </c>
+      <c r="E33">
+        <v>158.35218978102191</v>
+      </c>
+      <c r="F33">
+        <v>145.67883211678833</v>
+      </c>
+      <c r="G33">
+        <v>173.37472766884531</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D36" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E36" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F36" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G36" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H36" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I36" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J36" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K36" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L36" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M36" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N36" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>104.33581435956961</v>
+      </c>
+      <c r="D37">
+        <v>146.04090449018662</v>
+      </c>
+      <c r="E37">
+        <v>168.64785777600457</v>
+      </c>
+      <c r="F37">
+        <v>138.62529464674051</v>
+      </c>
+      <c r="G37">
+        <v>123.4988771545007</v>
+      </c>
+      <c r="H37">
+        <v>115.70093851436737</v>
+      </c>
+      <c r="I37">
+        <v>141.33336723596298</v>
+      </c>
+      <c r="J37">
+        <v>106.0351458617703</v>
+      </c>
+      <c r="K37">
+        <v>77.138510637832439</v>
+      </c>
+      <c r="L37">
+        <v>89.875493814747912</v>
+      </c>
+      <c r="M37">
+        <v>69.408167736869757</v>
+      </c>
+      <c r="N37">
+        <v>78.402152343025207</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>65.487783595113441</v>
+      </c>
+      <c r="D38">
+        <v>98.40789473684211</v>
+      </c>
+      <c r="E38">
+        <v>79.761278195488728</v>
+      </c>
+      <c r="F38">
+        <v>48.903601694915253</v>
+      </c>
+      <c r="G38">
+        <v>106.04545454545455</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D41" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E41" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F41" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G41" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H41" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I41" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J41" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K41" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L41" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M41" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N41" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
+        <v>0</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>87.669852578999993</v>
+      </c>
+      <c r="K42">
+        <v>106.0290884755</v>
+      </c>
+      <c r="L42">
+        <v>120.70637673100002</v>
+      </c>
+      <c r="M42">
+        <v>148.54745688599999</v>
+      </c>
+      <c r="N42">
+        <v>153.41811429099999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46143</v>
+      </c>
+      <c r="E46" s="1">
+        <v>46174</v>
+      </c>
+      <c r="F46" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G46" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H46" s="1">
+        <v>46266</v>
+      </c>
+      <c r="I46" s="1">
+        <v>46296</v>
+      </c>
+      <c r="J46" s="1">
+        <v>46327</v>
+      </c>
+      <c r="K46" s="1">
+        <v>46357</v>
+      </c>
+      <c r="L46" s="1">
+        <v>46388</v>
+      </c>
+      <c r="M46" s="1">
+        <v>46419</v>
+      </c>
+      <c r="N46" s="1">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>11</v>
+      </c>
+      <c r="B47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47">
+        <v>1068.6547450589999</v>
+      </c>
+      <c r="D47">
+        <v>522.72121195950001</v>
+      </c>
+      <c r="E47">
+        <v>527.11591197716677</v>
+      </c>
+      <c r="F47">
+        <v>289.89443335494997</v>
+      </c>
+      <c r="G47">
+        <v>1001.0243530167003</v>
+      </c>
+      <c r="H47">
+        <v>474.33255916849993</v>
+      </c>
+      <c r="I47">
+        <v>716.91005945537518</v>
+      </c>
+      <c r="J47">
+        <v>625.71999646492861</v>
+      </c>
+      <c r="K47">
+        <v>468.91274100912494</v>
+      </c>
+      <c r="L47">
+        <v>549.13499065230008</v>
+      </c>
+      <c r="M47">
+        <v>719.57935050575009</v>
+      </c>
+      <c r="N47">
+        <v>909.90780835316696</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>11</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48">
+        <v>976.60683760683764</v>
+      </c>
+      <c r="D48">
+        <v>2511.695652173913</v>
+      </c>
+      <c r="E48">
+        <v>2744.0614035087719</v>
+      </c>
+      <c r="F48">
+        <v>1122.5745856353592</v>
+      </c>
+      <c r="G48">
+        <v>664.15949367088604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>